<commit_message>
Assembly 4C — SPLT 2025 verified: +$68,855 confirmed, CB interco found
Four-point verification of the +$68,855 SPLT 2025 figure:
- FB invoice $97,769.11 confirmed via proper CSV parse (prior $85,325 was
  thousands-comma parser bug — documented as standing trap)
- ···3247 Chase FB $51,294.89 matches packet Section C exactly
- ···2100 WF debit: $1,134.82 bank-vs-invoice delta flagged for owner ID
- Chase charges-vs-payments gap $27,760 fully explained (no missing deductions)

New interco finding: CB 2025 FB invoice ($17,818.73) is ALL on SPLT Chase
···3247 — CB paid zero FB ads from its own bank. SPLT advanced the payment.
Treatment: SPLT receivable / CB payable + CB deduction $17,818.73. Zero SPLT
P&L impact. Feeds CB 2025 packet (next).

Updated: SPLT packet (Tab 5 ···2100 flag, Tab 6 interco, Tab 1 summary),
cover memo (Assembly 4C section), CLAUDE.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Downloads/Splitflask-Financials/deliverables/SPLT_2025_Amendment_Packet.xlsx
+++ b/Downloads/Splitflask-Financials/deliverables/SPLT_2025_Amendment_Packet.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -596,6 +596,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -950,6 +951,48 @@
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>• Corrected Amazon 1099-K from Amazon: Request corrected 1099-K from Amazon under SPLT TIN (EIN 33-3094308) as belt-and-suspenders. Does not change nominee treatment but reduces future inquiry risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <f>== ASSEMBLY 4C VERIFICATION FINDINGS (2026-07-11) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>FB Invoice Reconciliation</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Invoice total $97,769.11 CONFIRMED (proper CSV parse). ···3247 $51,294.89 ✓ matches Section C. ···2100 bank $22,351.63 vs invoice $21,216.81 → $1,134.82 flag (Tab 5 note added). No double-count between Sections B and C. CB 2025 FB invoice ($17,818.73 ALL on ···3247) = interco item → Tab 6 updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Chase charges-vs-payments</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>WF→Chase payments $118,406, Section C charges $90,646. Gap $27,760 = CB interco ads $17,819 + flagged items $6,080 + residual $3,861 (personal/timing). Gap fully explained — no missing SPLT deductions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Final number status</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>+$68,855 CONFIRMED internally consistent. Range: +$62,775 (all 6 flagged Chase items business) to +$69,990 (···2100 $1,134.82 non-Splitflask). Base case $68,855 stands pending owner IDs.</t>
         </is>
       </c>
     </row>
@@ -1854,6 +1897,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2192,7 +2236,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Debit card ···2100 charges IN WF bank statements. SEPARATE from Chase ···3247 credit card in Section C — no double-count.</t>
+          <t>Debit card ···2100 charges IN WF bank statements. SEPARATE from Chase ···3247 credit card in Section C — no double-count. ⚠️ ASSEMBLY 4C FLAG: Bank total $22,351.63 vs Splitflask FB invoice ···2100 $21,216.81 = $1,134.82 delta. Per CLAUDE.md rule, bank is authoritative for debit cards. However, $1,134.82 is NOT on the Splitflask invoice and NOT on the CB invoice (CB invoice = ···3247 only). Owner: confirm which Meta ad account the extra $1,134.82 belongs to (2nd Meta account? period overlap?). If non-Splitflask: remove $1,134.82 → income +$69,990. Currently using bank figure pending ID.</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2629,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Stated from Meta invoice. Card ···3247 = SPLT Chase card. Jan–Mar 2025 = Shark Tank airing period (heavy spend). SEPARATE from WF debit ···2100 (Section B) — no double-count.</t>
+          <t>Stated from Meta invoice. Card ···3247 = SPLT Chase card. Jan–Mar 2025 = Shark Tank airing period (heavy spend). SEPARATE from WF debit ···2100 (Section B) — no double-count. ⚠️ ASSEMBLY 4C FLAG: Bank total $22,351.63 vs Splitflask FB invoice ···2100 $21,216.81 = $1,134.82 delta. Per CLAUDE.md rule, bank is authoritative for debit cards. However, $1,134.82 is NOT on the Splitflask invoice and NOT on the CB invoice (CB invoice = ···3247 only). Owner: confirm which Meta ad account the extra $1,134.82 belongs to (2nd Meta account? period overlap?). If non-Splitflask: remove $1,134.82 → income +$69,990. Currently using bank figure pending ID.</t>
         </is>
       </c>
     </row>
@@ -2890,6 +2934,7 @@
       </c>
     </row>
     <row r="51" ht="42" customHeight="1"/>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="6" t="n"/>
@@ -2921,6 +2966,7 @@
         <v/>
       </c>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
@@ -2945,6 +2991,7 @@
         <v/>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="22" t="inlineStr">
         <is>
@@ -3159,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3182,6 +3229,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -3432,22 +3480,44 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>SPLT↔CB</t>
+          <t>SPLT→CB via Chase ···3247 (NEW — Assembly 4C finding)</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>$0 confirmed</t>
+          <t>SPLT paid CB FB ads $17,818.73 via ···3247</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>No interco flows</t>
+          <t>⚠️ INTERCO RECEIVABLE — balance sheet, NOT P&amp;L on SPLT</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Layer 10 verified: zero SPLT↔CB interco transactions in either entity's 2025 statements. PASS.</t>
+          <t>CB 2025 FB invoice (Meta ad account for Cyberbrands) shows ALL $17,818.73 charged to ···3247 (SPLT Chase card). CB paid ZERO of its own FB ads from CB bank. SPLT advanced the payment. Treatment: SPLT records interco receivable $17,818.73 (CB owes SPLT); CB records payable $17,818.73 + FB ad DEDUCTION $17,818.73. Zero P&amp;L impact on SPLT. FEEDS CB 2025 PACKET. Layer 10 SPLT↔CB=$0 was correct for WF bank flows only — Chase card flows were not in scope then.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>⚠️ CB 2025 action: deduct $17,818.73 FB ads (paid by SPLT on CB behalf)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>$17,818.73</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CB 2025 DEDUCTION — in CB 2025 packet</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Layer 10 was bank-only; Chase card flows discovered in Assembly 4C. CB 2025 packet must add $17,818.73 FB ads from SPLT Chase interco as CB deduction. Cross-check: SPLT receivable $17,818.73 = CB payable $17,818.73.</t>
         </is>
       </c>
     </row>

</xml_diff>